<commit_message>
Record user-reported live tests and clear recovered email errors
</commit_message>
<xml_diff>
--- a/submission/Allo_Operations_Template.xlsx
+++ b/submission/Allo_Operations_Template.xlsx
@@ -490,7 +490,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Template and local tests supplied; live Google authorization and email receipts pending.</t>
+          <t>Template/local tests supplied; core live workflow and email tests reported by user. See HOSTED_ACCEPTANCE.md.</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Completion anchored: +7/15/30 calendar days. Daily: next Monday–Friday. Holidays not modeled.</t>
+          <t>Completion anchored: +7/15/30 calendar days. Daily: next Mondayâ€“Friday. Holidays not modeled.</t>
         </is>
       </c>
     </row>
@@ -658,7 +658,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>29/29 tests passed; all 8 deterministic scenarios passed. These use local adapters.</t>
+          <t>30/30 tests passed; all 8 deterministic scenarios passed. These use local adapters.</t>
         </is>
       </c>
     </row>

</xml_diff>